<commit_message>
chore: update skills collection (3885 skills)
</commit_message>
<xml_diff>
--- a/skills/antigravity-second-deposit-igaming/examples/export-example.xlsx
+++ b/skills/antigravity-second-deposit-igaming/examples/export-example.xlsx
@@ -143,7 +143,7 @@
   <sheetPr>
     <tabColor rgb="FFFFB800"/>
   </sheetPr>
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -165,219 +165,231 @@
       </c>
     </row>
     <row r="3"/>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+    <row r="4" ht="64" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ограничения</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Описательные гипотезы, не причины и не доказанный эффект. Правила стран — непроверенный снимок; подтвердите применимость. Список контактов по умолчанию отключен: нужны проверка возраста, согласия, RG и явное включение оператором.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">Когда смотреть</t>
         </is>
       </c>
-      <c r="B4" s="11"/>
-    </row>
-    <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Первый запуск</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Выгрузка за 60-120 дней по сегодняшний день. Скилл считает норму, недобор вторых депозитов и показатели по FTD старше 7 дней и сохраняет базу. Повторять раз в месяц.</t>
-        </is>
-      </c>
+      <c r="B5" s="11"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Каждый день</t>
+          <t xml:space="preserve">Первый запуск</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Выгрузка за последние 7 дней, у игроков дата первого депозита. Скилл собирает список на сегодня по FTD за 72 часа: кому писать сейчас и что предложить, файл на каждое действие для CRM. Способы оплаты и история причин берутся из базы. Запуск можно поставить по расписанию: выгрузки кладутся в одну папку, скилл берет самую свежую.</t>
+          <t xml:space="preserve">Выгрузка за 60-120 дней по сегодняшний день. Скилл считает норму, недобор вторых депозитов и показатели по FTD старше 7 дней и сохраняет базу. Повторять раз в месяц.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Каждый день</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выгрузка за последние 7 дней, у игроков дата первого депозита. Скилл собирает список на сегодня по FTD за 72 часа: кому писать сейчас и что предложить, файл на каждое действие для CRM. Способы оплаты и история причин берутся из базы. Запуск можно поставить по расписанию: выгрузки кладутся в одну папку, скилл берет самую свежую.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Контрольная группа</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">20% списка не получают сообщений 7 дней (сервисные случаи всегда получают помощь). Скилл ведет журнал и показывает, на сколько чаще возвращаются те, кому писали.</t>
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+    <row r="9"/>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">Когда виден сигнал</t>
         </is>
       </c>
-      <c r="B9" s="11"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Много отказов подряд</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Сразу после третьего отказа за 30 минут. Сейчас личное сообщение или звонок саппорта.</t>
-        </is>
-      </c>
+      <c r="B10" s="11"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Второй депозит не прошел</t>
+          <t xml:space="preserve">Много отказов подряд</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сразу после отказа в кассе. В течение 15 минут другой способ оплаты.</t>
+          <t xml:space="preserve">Сразу после третьего отказа за 30 минут. Сейчас личное сообщение или звонок саппорта.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вывод отклонен</t>
+          <t xml:space="preserve">Второй депозит не прошел</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">В момент отказа по выводу. Сразу саппорт: причина и что сделать.</t>
+          <t xml:space="preserve">Сразу после отказа в кассе. В течение 15 минут другой способ оплаты.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Запросили документы</t>
+          <t xml:space="preserve">Вывод отклонен</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">В момент запроса проверки. Помочь пройти проверку.</t>
+          <t xml:space="preserve">В момент отказа по выводу. Сразу саппорт: причина и что сделать.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Отыграл бонус и вывел</t>
+          <t xml:space="preserve">Запросили документы</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">В момент запроса вывода. Новых депозитных бонусов не давать.</t>
+          <t xml:space="preserve">В момент запроса проверки. Помочь пройти проверку.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Долгий вывод</t>
+          <t xml:space="preserve">Отыграл бонус и вывел</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Через 24 часа после запроса, если вывод не выплачен, или раньше, если закон страны требует быстрее (Бразилия 2 часа, Колумбия 12). Провести и сообщить срок.</t>
+          <t xml:space="preserve">В момент запроса вывода. Новых депозитных бонусов не давать.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Выиграл и вывел</t>
+          <t xml:space="preserve">Долгий вывод</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">В момент запроса вывода. В обработке: провести быстро. Выплачен: через 2-3 дня повод вернуться.</t>
+          <t xml:space="preserve">Через 24 часа после запроса, если вывод не выплачен, или раньше, если закон страны требует быстрее (Бразилия 2 часа, Колумбия 12). Провести и сообщить срок.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бонус с тяжелым вейджером</t>
+          <t xml:space="preserve">Выиграл и вывел</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">В момент FTD. Отыгрывается: напомнить о прогрессе. Проигран: оффер без тяжелого вейджера.</t>
+          <t xml:space="preserve">В момент запроса вывода. В обработке: провести быстро. Выплачен: через 2-3 дня повод вернуться.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сгорел быстро</t>
+          <t xml:space="preserve">Бонус с тяжелым вейджером</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">В первую сессию. В течение 24 часов, без давления на депозит.</t>
+          <t xml:space="preserve">В момент FTD. Отыгрывается: напомнить о прогрессе. Проигран: оффер без тяжелого вейджера.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Выиграл и не вывел</t>
+          <t xml:space="preserve">Сгорел быстро</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Через 24 часа после FTD. Поздравить и дать повод играть дальше.</t>
+          <t xml:space="preserve">В первую сессию. В течение 24 часов, без давления на депозит.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Деньги на балансе</t>
+          <t xml:space="preserve">Выиграл и не вывел</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Через 24 часа после FTD. Напомнить про баланс.</t>
+          <t xml:space="preserve">Через 24 часа после FTD. Поздравить и дать повод играть дальше.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Деньги на балансе</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Через 24 часа после FTD. Напомнить про баланс.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">FTD не с первой попытки</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">В момент FTD. Кнопка со способом, который прошел, в сообщении о втором депозите.</t>
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+    <row r="23"/>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">Какие листы нужны</t>
         </is>
       </c>
-      <c r="B23" s="11"/>
-    </row>
-    <row r="24" ht="64" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="B24" s="11"/>
+    </row>
+    <row r="25" ht="64" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Депозиты (обязательно)</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Все попытки депозита за 60-120 дней: успешные, отклоненные, брошенные.
 Где взять: отчет по платежам или транзакциям: тип Deposit, все статусы.
@@ -385,13 +397,13 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="64" customHeight="1">
-      <c r="A25" s="8" t="inlineStr">
+    <row r="26" ht="64" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Выводы (желательно)</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Запросы на вывод за тот же период.
 Где взять: тот же отчет по транзакциям: тип Withdrawal.
@@ -399,13 +411,13 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="64" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
+    <row r="27" ht="64" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Бонусы (желательно)</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Начисленные бонусы с вейджером.
 Где взять: отчет по бонусам.
@@ -413,13 +425,13 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="64" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
+    <row r="28" ht="64" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Ставки (желательно)</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Ставки и выигрыши реальными деньгами по игроку за день или за сессию.
 Где взять: отчет по игровой активности или GGR по игрокам с разбивкой по дням.
@@ -427,13 +439,13 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="64" customHeight="1">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="29" ht="64" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Игроки (желательно)</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Дата регистрации, страна, источник, флаги ответственной игры.
 Где взять: список игроков.
@@ -441,303 +453,303 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
+    <row r="30"/>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">Правила</t>
         </is>
       </c>
-      <c r="B30" s="11"/>
-    </row>
-    <row r="31" ht="32" customHeight="1">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Период</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Первый запуск и раз в месяц: 60-120 дней по сегодняшний день. Каждый день: последние 7 дней с датой первого депозита у игроков.</t>
-        </is>
-      </c>
+      <c r="B31" s="11"/>
     </row>
     <row r="32" ht="32" customHeight="1">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Все попытки</t>
+          <t xml:space="preserve">Период</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Депозиты нужны со всеми статусами, включая отклоненные и брошенные. Без них сценарий "Второй депозит не прошел" не посчитается.</t>
+          <t xml:space="preserve">Первый запуск и раз в месяц: 60-120 дней по сегодняшний день. Каждый день: последние 7 дней с датой первого депозита у игроков.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="32" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Без личных данных</t>
+          <t xml:space="preserve">Все попытки</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Нужен только ID игрока, одинаковый во всех листах. Имена, email, телефоны и адреса не выгружайте.</t>
+          <t xml:space="preserve">Депозиты нужны со всеми статусами, включая отклоненные и брошенные. Без них сценарий "Второй депозит не прошел" не посчитается.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="32" customHeight="1">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Свои названия</t>
+          <t xml:space="preserve">Без личных данных</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Колонки и статусы могут называться как угодно, листы могут лежать отдельными файлами CSV или XLSX. Скилл сопоставит их сам и спросит, если статус непонятен.</t>
+          <t xml:space="preserve">Нужен только ID игрока, одинаковый во всех листах. Имена, email, телефоны и адреса не выгружайте.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="32" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Даты и время</t>
+          <t xml:space="preserve">Свои названия</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Любой формат. Время во всех файлах в одном часовом поясе, лучше UTC.</t>
+          <t xml:space="preserve">Колонки и статусы могут называться как угодно, листы могут лежать отдельными файлами CSV или XLSX. Скилл сопоставит их сам и спросит, если статус непонятен.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="32" customHeight="1">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Валюта</t>
+          <t xml:space="preserve">Даты и время</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Если валют несколько, добавьте колонку валюты: скилл спросит курс к валюте отчета.</t>
+          <t xml:space="preserve">Поддерживаемые форматы; неоднозначные даты и разделитель задайте явно. Время во всех файлах в одном часовом поясе, лучше UTC.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="32" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Страна</t>
+          <t xml:space="preserve">Валюта</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Код страны игрока (BR, DE, GB) включает правила стран: законный срок выплаты, запрещенные способы оплаты, законные лимиты депозитов.</t>
+          <t xml:space="preserve">Если валют несколько, добавьте колонку валюты: скилл спросит курс к валюте отчета.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="32" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Google Таблицы</t>
+          <t xml:space="preserve">Страна</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Файл, Скачать, Microsoft Excel (.xlsx): все листы попадут в один файл. По ссылке скилл таблицы не читает, чтобы данные игроков не были открыты всем, у кого есть ссылка.</t>
+          <t xml:space="preserve">Код страны игрока (BR, DE, GB) включает правила стран: законный срок выплаты, запрещенные способы оплаты, законные лимиты депозитов.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="32" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Google Таблицы</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Файл, Скачать, Microsoft Excel (.xlsx): все листы попадут в один файл. По ссылке скилл таблицы не читает, чтобы данные игроков не были открыты всем, у кого есть ссылка.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">SQL для аналитика</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Готовые запросы на каждый лист и минимальный вариант одним запросом: examples/export-queries.sql в папке скилла. Названия колонок в них те же, что здесь.</t>
         </is>
       </c>
     </row>
-    <row r="40"/>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="11" t="inlineStr">
+    <row r="41"/>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">Кто есть кто в примере</t>
         </is>
       </c>
-      <c r="B41" s="11"/>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">100231</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Обычный игрок: FTD 50 €, через два дня второй депозит, потом третий.</t>
-        </is>
-      </c>
+      <c r="B42" s="11"/>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100232</t>
+          <t xml:space="preserve">100231</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Второй депозит не прошел: две попытки картой отклонены, игрок ушел.</t>
+          <t xml:space="preserve">Обычный игрок: FTD 50 €, через два дня второй депозит, потом третий.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100233</t>
+          <t xml:space="preserve">100232</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сгорел быстро: поставил 60 € с депозита 20 € крупными спинами и проиграл 92%.</t>
+          <t xml:space="preserve">Второй депозит не прошел: две попытки картой отклонены, игрок ушел.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100234</t>
+          <t xml:space="preserve">100233</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бонус с тяжелым вейджером: к FTD 100 € взял Welcome 100% x40.</t>
+          <t xml:space="preserve">Сгорел быстро: поставил 60 € с депозита 20 € крупными спинами и проиграл 92%.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100235</t>
+          <t xml:space="preserve">100234</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Выиграл и вывел: внес 50 €, на следующий день вывел 180 €.</t>
+          <t xml:space="preserve">Бонус с тяжелым вейджером: к FTD 100 € взял Welcome 100% x40.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100236</t>
+          <t xml:space="preserve">100235</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Деньги на балансе: внес 100 €, поставил 15 € и пропал.</t>
+          <t xml:space="preserve">Выиграл и вывел: внес 50 €, на следующий день вывел 180 €.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100237</t>
+          <t xml:space="preserve">100236</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Самоисключение: не попадет ни в расчет, ни в список.</t>
+          <t xml:space="preserve">Деньги на балансе: внес 100 €, поставил 15 € и пропал.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100238</t>
+          <t xml:space="preserve">100237</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">FTD не с первой попытки: бросил оплату картой, внес другим способом, потом вернулся.</t>
+          <t xml:space="preserve">Самоисключение: не попадет ни в расчет, ни в список.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100239</t>
+          <t xml:space="preserve">100238</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Много отказов подряд: после FTD три отказа картой за 7 минут.</t>
+          <t xml:space="preserve">FTD не с первой попытки: бросил оплату картой, внес другим способом, потом вернулся.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100240</t>
+          <t xml:space="preserve">100239</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вывод отклонен: запросил вывод 120 €, отказ.</t>
+          <t xml:space="preserve">Много отказов подряд: после FTD три отказа картой за 7 минут.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100241</t>
+          <t xml:space="preserve">100240</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Запросили документы: через 20 часов после FTD, второго депозита нет.</t>
+          <t xml:space="preserve">Вывод отклонен: запросил вывод 120 €, отказ.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100242</t>
+          <t xml:space="preserve">100241</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Отыграл бонус и вывел: взял Welcome 100% x40, вывел 260 €.</t>
+          <t xml:space="preserve">Запросили документы: через 20 часов после FTD, второго депозита нет.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100243</t>
+          <t xml:space="preserve">100242</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Долгий вывод: запрос 11.10, выплата через 52 часа.</t>
+          <t xml:space="preserve">Отыграл бонус и вывел: взял Welcome 100% x40, вывел 260 €.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">100243</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Долгий вывод: запрос 11.10, выплата через 52 часа.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">100244</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Выиграл и не вывел: внес 50 €, выиграл 95 € и пропал.</t>
         </is>
       </c>
     </row>
-    <row r="56"/>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="7" t="inlineStr">
+    <row r="57"/>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Описание каждой колонки на листе "Колонки". Отчет и список игроков скилл соберет сам.</t>
         </is>
@@ -747,7 +759,7 @@
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A58:B58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>